<commit_message>
alterações e melhorias projeto excel voice
</commit_message>
<xml_diff>
--- a/ExcelVoice/ETP.xlsx
+++ b/ExcelVoice/ETP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\Desktop\IM\IM_EXCEL_NODEPENDENCIES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\Desktop\IM\IM_EXCEL_Projects\ExcelVoice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16D08DC-8317-4101-B24D-211F09581E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAA35A1-BE1A-458F-B1C9-6FA75737BB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="14112" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1635,7 +1635,10 @@
       <c r="N2" s="5">
         <v>15</v>
       </c>
-      <c r="O2" s="6"/>
+      <c r="O2" s="6">
+        <f>AVERAGE(H2,N2)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
@@ -1680,7 +1683,10 @@
       <c r="N3" s="8">
         <v>11</v>
       </c>
-      <c r="O3" s="8"/>
+      <c r="O3" s="8">
+        <f>AVERAGE(H3,N3)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
@@ -1725,7 +1731,10 @@
       <c r="N4" s="1">
         <v>10</v>
       </c>
-      <c r="O4" s="1"/>
+      <c r="O4" s="1">
+        <f>AVERAGE(H4,N4)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
@@ -1766,7 +1775,10 @@
       <c r="N5" s="8">
         <v>19</v>
       </c>
-      <c r="O5" s="8"/>
+      <c r="O5" s="8">
+        <f>AVERAGE(H5,N5)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
@@ -1811,7 +1823,10 @@
       <c r="N6" s="1">
         <v>7</v>
       </c>
-      <c r="O6" s="1"/>
+      <c r="O6" s="1">
+        <f>AVERAGE(H6,N6)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
@@ -1856,7 +1871,10 @@
       <c r="N7" s="8">
         <v>11</v>
       </c>
-      <c r="O7" s="8"/>
+      <c r="O7" s="8">
+        <f>AVERAGE(H7,N7)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
@@ -1901,7 +1919,10 @@
       <c r="N8" s="1">
         <v>10</v>
       </c>
-      <c r="O8" s="1"/>
+      <c r="O8" s="1">
+        <f>AVERAGE(H8,N8)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
@@ -1946,7 +1967,10 @@
       <c r="N9" s="8">
         <v>18</v>
       </c>
-      <c r="O9" s="8"/>
+      <c r="O9" s="8">
+        <f>AVERAGE(H9,N9)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
@@ -1991,7 +2015,10 @@
       <c r="N10" s="1">
         <v>19</v>
       </c>
-      <c r="O10" s="1"/>
+      <c r="O10" s="1">
+        <f>AVERAGE(H10,N10)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="7">
@@ -2036,7 +2063,10 @@
       <c r="N11" s="8">
         <v>13</v>
       </c>
-      <c r="O11" s="8"/>
+      <c r="O11" s="8">
+        <f>AVERAGE(H11,N11)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
@@ -2081,7 +2111,10 @@
       <c r="N12" s="1">
         <v>16</v>
       </c>
-      <c r="O12" s="1"/>
+      <c r="O12" s="1">
+        <f>AVERAGE(H12,N12)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="7">
@@ -2126,7 +2159,10 @@
       <c r="N13" s="8">
         <v>18</v>
       </c>
-      <c r="O13" s="8"/>
+      <c r="O13" s="8">
+        <f>AVERAGE(H13,N13)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
@@ -2171,7 +2207,10 @@
       <c r="N14" s="1">
         <v>15</v>
       </c>
-      <c r="O14" s="1"/>
+      <c r="O14" s="1">
+        <f>AVERAGE(H14,N14)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
@@ -2216,7 +2255,10 @@
       <c r="N15" s="8">
         <v>7</v>
       </c>
-      <c r="O15" s="8"/>
+      <c r="O15" s="8">
+        <f>AVERAGE(H15,N15)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
@@ -2261,7 +2303,10 @@
       <c r="N16" s="1">
         <v>15</v>
       </c>
-      <c r="O16" s="1"/>
+      <c r="O16" s="1">
+        <f>AVERAGE(H16,N16)</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
@@ -2306,7 +2351,10 @@
       <c r="N17" s="8">
         <v>12</v>
       </c>
-      <c r="O17" s="8"/>
+      <c r="O17" s="8">
+        <f>AVERAGE(H17,N17)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
@@ -2351,7 +2399,10 @@
       <c r="N18" s="1">
         <v>16</v>
       </c>
-      <c r="O18" s="1"/>
+      <c r="O18" s="1">
+        <f>AVERAGE(H18,N18)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="7">
@@ -2396,7 +2447,10 @@
       <c r="N19" s="8">
         <v>7</v>
       </c>
-      <c r="O19" s="8"/>
+      <c r="O19" s="8">
+        <f>AVERAGE(H19,N19)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
@@ -2441,7 +2495,10 @@
       <c r="N20" s="1">
         <v>19</v>
       </c>
-      <c r="O20" s="1"/>
+      <c r="O20" s="1">
+        <f>AVERAGE(H20,N20)</f>
+        <v>17</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
@@ -2486,7 +2543,10 @@
       <c r="N21" s="8">
         <v>16</v>
       </c>
-      <c r="O21" s="8"/>
+      <c r="O21" s="8">
+        <f>AVERAGE(H21,N21)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
@@ -2531,7 +2591,10 @@
       <c r="N22" s="1">
         <v>13</v>
       </c>
-      <c r="O22" s="1"/>
+      <c r="O22" s="1">
+        <f>AVERAGE(H22,N22)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="7">
@@ -2576,7 +2639,10 @@
       <c r="N23" s="8">
         <v>12</v>
       </c>
-      <c r="O23" s="8"/>
+      <c r="O23" s="8">
+        <f>AVERAGE(H23,N23)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
@@ -2621,7 +2687,10 @@
       <c r="N24" s="1">
         <v>10</v>
       </c>
-      <c r="O24" s="1"/>
+      <c r="O24" s="1">
+        <f>AVERAGE(H24,N24)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="7">
@@ -2666,7 +2735,10 @@
       <c r="N25" s="8">
         <v>8</v>
       </c>
-      <c r="O25" s="8"/>
+      <c r="O25" s="8">
+        <f>AVERAGE(H25,N25)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
@@ -2711,7 +2783,10 @@
       <c r="N26" s="1">
         <v>15</v>
       </c>
-      <c r="O26" s="1"/>
+      <c r="O26" s="1">
+        <f>AVERAGE(H26,N26)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="7">
@@ -2756,7 +2831,10 @@
       <c r="N27" s="8">
         <v>7</v>
       </c>
-      <c r="O27" s="8"/>
+      <c r="O27" s="8">
+        <f>AVERAGE(H27,N27)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
@@ -2801,7 +2879,10 @@
       <c r="N28" s="1">
         <v>11</v>
       </c>
-      <c r="O28" s="1"/>
+      <c r="O28" s="1">
+        <f>AVERAGE(H28,N28)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="7">
@@ -2846,7 +2927,10 @@
       <c r="N29" s="8">
         <v>18</v>
       </c>
-      <c r="O29" s="8"/>
+      <c r="O29" s="8">
+        <f>AVERAGE(H29,N29)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
@@ -2891,7 +2975,10 @@
       <c r="N30" s="1">
         <v>18</v>
       </c>
-      <c r="O30" s="1"/>
+      <c r="O30" s="1">
+        <f>AVERAGE(H30,N30)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="7">
@@ -2936,7 +3023,10 @@
       <c r="N31" s="8">
         <v>16</v>
       </c>
-      <c r="O31" s="8"/>
+      <c r="O31" s="8">
+        <f>AVERAGE(H31,N31)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="9">
@@ -2981,7 +3071,10 @@
       <c r="N32" s="1">
         <v>13</v>
       </c>
-      <c r="O32" s="1"/>
+      <c r="O32" s="1">
+        <f>AVERAGE(H32,N32)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="7">
@@ -3026,7 +3119,10 @@
       <c r="N33" s="8">
         <v>12</v>
       </c>
-      <c r="O33" s="8"/>
+      <c r="O33" s="8">
+        <f>AVERAGE(H33,N33)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="9">
@@ -3071,7 +3167,10 @@
       <c r="N34" s="1">
         <v>14</v>
       </c>
-      <c r="O34" s="1"/>
+      <c r="O34" s="1">
+        <f>AVERAGE(H34,N34)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="7">
@@ -3116,7 +3215,10 @@
       <c r="N35" s="8">
         <v>15</v>
       </c>
-      <c r="O35" s="8"/>
+      <c r="O35" s="8">
+        <f>AVERAGE(H35,N35)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="9">
@@ -3161,7 +3263,10 @@
       <c r="N36" s="1">
         <v>15</v>
       </c>
-      <c r="O36" s="1"/>
+      <c r="O36" s="1">
+        <f>AVERAGE(H36,N36)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="7">
@@ -3206,7 +3311,10 @@
       <c r="N37" s="8">
         <v>16</v>
       </c>
-      <c r="O37" s="8"/>
+      <c r="O37" s="8">
+        <f>AVERAGE(H37,N37)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="9">
@@ -3251,7 +3359,10 @@
       <c r="N38" s="1">
         <v>9</v>
       </c>
-      <c r="O38" s="1"/>
+      <c r="O38" s="1">
+        <f>AVERAGE(H38,N38)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="7">
@@ -3296,7 +3407,10 @@
       <c r="N39" s="8">
         <v>15</v>
       </c>
-      <c r="O39" s="8"/>
+      <c r="O39" s="8">
+        <f>AVERAGE(H39,N39)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="9">
@@ -3341,7 +3455,10 @@
       <c r="N40" s="1">
         <v>13</v>
       </c>
-      <c r="O40" s="1"/>
+      <c r="O40" s="1">
+        <f>AVERAGE(H40,N40)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="7">
@@ -3386,7 +3503,10 @@
       <c r="N41" s="8">
         <v>18</v>
       </c>
-      <c r="O41" s="8"/>
+      <c r="O41" s="8">
+        <f>AVERAGE(H41,N41)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="9">
@@ -3431,7 +3551,10 @@
       <c r="N42" s="1">
         <v>13</v>
       </c>
-      <c r="O42" s="1"/>
+      <c r="O42" s="1">
+        <f>AVERAGE(H42,N42)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="7">
@@ -3476,7 +3599,10 @@
       <c r="N43" s="8">
         <v>16</v>
       </c>
-      <c r="O43" s="8"/>
+      <c r="O43" s="8">
+        <f>AVERAGE(H43,N43)</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="9">
@@ -3521,7 +3647,10 @@
       <c r="N44" s="1">
         <v>8</v>
       </c>
-      <c r="O44" s="1"/>
+      <c r="O44" s="1">
+        <f>AVERAGE(H44,N44)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="7">
@@ -3566,7 +3695,10 @@
       <c r="N45" s="8">
         <v>13</v>
       </c>
-      <c r="O45" s="8"/>
+      <c r="O45" s="8">
+        <f>AVERAGE(H45,N45)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="9">
@@ -3611,7 +3743,10 @@
       <c r="N46" s="1">
         <v>19</v>
       </c>
-      <c r="O46" s="1"/>
+      <c r="O46" s="1">
+        <f>AVERAGE(H46,N46)</f>
+        <v>18.5</v>
+      </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="7">
@@ -3656,7 +3791,10 @@
       <c r="N47" s="8">
         <v>15</v>
       </c>
-      <c r="O47" s="8"/>
+      <c r="O47" s="8">
+        <f>AVERAGE(H47,N47)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="9">
@@ -3701,7 +3839,10 @@
       <c r="N48" s="1">
         <v>15</v>
       </c>
-      <c r="O48" s="1"/>
+      <c r="O48" s="1">
+        <f>AVERAGE(H48,N48)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="7">
@@ -3746,7 +3887,10 @@
       <c r="N49" s="8">
         <v>10</v>
       </c>
-      <c r="O49" s="8"/>
+      <c r="O49" s="8">
+        <f>AVERAGE(H49,N49)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="9">
@@ -3791,7 +3935,10 @@
       <c r="N50" s="1">
         <v>9</v>
       </c>
-      <c r="O50" s="1"/>
+      <c r="O50" s="1">
+        <f>AVERAGE(H50,N50)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="7">
@@ -3836,7 +3983,10 @@
       <c r="N51" s="8">
         <v>10</v>
       </c>
-      <c r="O51" s="8"/>
+      <c r="O51" s="8">
+        <f>AVERAGE(H51,N51)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="9">
@@ -3881,7 +4031,10 @@
       <c r="N52" s="1">
         <v>17</v>
       </c>
-      <c r="O52" s="1"/>
+      <c r="O52" s="1">
+        <f>AVERAGE(H52,N52)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="7">
@@ -3926,7 +4079,10 @@
       <c r="N53" s="8">
         <v>19</v>
       </c>
-      <c r="O53" s="8"/>
+      <c r="O53" s="8">
+        <f>AVERAGE(H53,N53)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="9">
@@ -3971,7 +4127,10 @@
       <c r="N54" s="1">
         <v>13</v>
       </c>
-      <c r="O54" s="1"/>
+      <c r="O54" s="1">
+        <f>AVERAGE(H54,N54)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="7">
@@ -4016,7 +4175,10 @@
       <c r="N55" s="8">
         <v>10</v>
       </c>
-      <c r="O55" s="8"/>
+      <c r="O55" s="8">
+        <f>AVERAGE(H55,N55)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="9">
@@ -4061,7 +4223,10 @@
       <c r="N56" s="1">
         <v>13</v>
       </c>
-      <c r="O56" s="1"/>
+      <c r="O56" s="1">
+        <f>AVERAGE(H56,N56)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="7">
@@ -4106,7 +4271,10 @@
       <c r="N57" s="8">
         <v>12</v>
       </c>
-      <c r="O57" s="8"/>
+      <c r="O57" s="8">
+        <f>AVERAGE(H57,N57)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="9">
@@ -4151,7 +4319,10 @@
       <c r="N58" s="1">
         <v>14</v>
       </c>
-      <c r="O58" s="1"/>
+      <c r="O58" s="1">
+        <f>AVERAGE(H58,N58)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="7">
@@ -4196,7 +4367,10 @@
       <c r="N59" s="8">
         <v>18</v>
       </c>
-      <c r="O59" s="8"/>
+      <c r="O59" s="8">
+        <f>AVERAGE(H59,N59)</f>
+        <v>17</v>
+      </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="9">
@@ -4241,7 +4415,10 @@
       <c r="N60" s="1">
         <v>7</v>
       </c>
-      <c r="O60" s="1"/>
+      <c r="O60" s="1">
+        <f>AVERAGE(H60,N60)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="7">
@@ -4286,7 +4463,10 @@
       <c r="N61" s="8">
         <v>18</v>
       </c>
-      <c r="O61" s="8"/>
+      <c r="O61" s="8">
+        <f>AVERAGE(H61,N61)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="9">
@@ -4331,7 +4511,10 @@
       <c r="N62" s="1">
         <v>15</v>
       </c>
-      <c r="O62" s="1"/>
+      <c r="O62" s="1">
+        <f>AVERAGE(H62,N62)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="7">
@@ -4376,7 +4559,10 @@
       <c r="N63" s="8">
         <v>11</v>
       </c>
-      <c r="O63" s="8"/>
+      <c r="O63" s="8">
+        <f>AVERAGE(H63,N63)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="9">
@@ -4421,7 +4607,10 @@
       <c r="N64" s="1">
         <v>17</v>
       </c>
-      <c r="O64" s="1"/>
+      <c r="O64" s="1">
+        <f>AVERAGE(H64,N64)</f>
+        <v>17.5</v>
+      </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="7">
@@ -4466,7 +4655,10 @@
       <c r="N65" s="8">
         <v>13</v>
       </c>
-      <c r="O65" s="8"/>
+      <c r="O65" s="8">
+        <f>AVERAGE(H65,N65)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="9">
@@ -4511,7 +4703,10 @@
       <c r="N66" s="1">
         <v>18</v>
       </c>
-      <c r="O66" s="1"/>
+      <c r="O66" s="1">
+        <f>AVERAGE(H66,N66)</f>
+        <v>17</v>
+      </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="7">
@@ -4556,7 +4751,10 @@
       <c r="N67" s="8">
         <v>12</v>
       </c>
-      <c r="O67" s="8"/>
+      <c r="O67" s="8">
+        <f>AVERAGE(H67,N67)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="9">
@@ -4601,7 +4799,10 @@
       <c r="N68" s="1">
         <v>19</v>
       </c>
-      <c r="O68" s="1"/>
+      <c r="O68" s="1">
+        <f>AVERAGE(H68,N68)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="7">
@@ -4646,7 +4847,10 @@
       <c r="N69" s="8">
         <v>15</v>
       </c>
-      <c r="O69" s="8"/>
+      <c r="O69" s="8">
+        <f>AVERAGE(H69,N69)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="9">
@@ -4691,7 +4895,10 @@
       <c r="N70" s="1">
         <v>9</v>
       </c>
-      <c r="O70" s="1"/>
+      <c r="O70" s="1">
+        <f>AVERAGE(H70,N70)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="7">
@@ -4736,7 +4943,10 @@
       <c r="N71" s="8">
         <v>18</v>
       </c>
-      <c r="O71" s="8"/>
+      <c r="O71" s="8">
+        <f>AVERAGE(H71,N71)</f>
+        <v>17.5</v>
+      </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="9">
@@ -4781,7 +4991,10 @@
       <c r="N72" s="1">
         <v>10</v>
       </c>
-      <c r="O72" s="1"/>
+      <c r="O72" s="1">
+        <f>AVERAGE(H72,N72)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="7">
@@ -4826,7 +5039,10 @@
       <c r="N73" s="8">
         <v>16</v>
       </c>
-      <c r="O73" s="8"/>
+      <c r="O73" s="8">
+        <f>AVERAGE(H73,N73)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="9">
@@ -4871,7 +5087,10 @@
       <c r="N74" s="1">
         <v>14</v>
       </c>
-      <c r="O74" s="1"/>
+      <c r="O74" s="1">
+        <f>AVERAGE(H74,N74)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75" s="7">
@@ -4916,7 +5135,10 @@
       <c r="N75" s="8">
         <v>12</v>
       </c>
-      <c r="O75" s="8"/>
+      <c r="O75" s="8">
+        <f>AVERAGE(H75,N75)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76" s="9">
@@ -4961,7 +5183,10 @@
       <c r="N76" s="1">
         <v>10</v>
       </c>
-      <c r="O76" s="1"/>
+      <c r="O76" s="1">
+        <f>AVERAGE(H76,N76)</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77" s="7">
@@ -5006,7 +5231,10 @@
       <c r="N77" s="8">
         <v>11</v>
       </c>
-      <c r="O77" s="8"/>
+      <c r="O77" s="8">
+        <f>AVERAGE(H77,N77)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="9">
@@ -5051,7 +5279,10 @@
       <c r="N78" s="1">
         <v>12</v>
       </c>
-      <c r="O78" s="1"/>
+      <c r="O78" s="1">
+        <f>AVERAGE(H78,N78)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79" s="7">
@@ -5096,7 +5327,10 @@
       <c r="N79" s="8">
         <v>10</v>
       </c>
-      <c r="O79" s="8"/>
+      <c r="O79" s="8">
+        <f>AVERAGE(H79,N79)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="9">
@@ -5141,7 +5375,10 @@
       <c r="N80" s="1">
         <v>10</v>
       </c>
-      <c r="O80" s="1"/>
+      <c r="O80" s="1">
+        <f>AVERAGE(H80,N80)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81" s="7">
@@ -5186,7 +5423,10 @@
       <c r="N81" s="8">
         <v>14</v>
       </c>
-      <c r="O81" s="8"/>
+      <c r="O81" s="8">
+        <f>AVERAGE(H81,N81)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82" s="9">
@@ -5231,7 +5471,10 @@
       <c r="N82" s="1">
         <v>16</v>
       </c>
-      <c r="O82" s="1"/>
+      <c r="O82" s="1">
+        <f>AVERAGE(H82,N82)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83" s="7">
@@ -5276,7 +5519,10 @@
       <c r="N83" s="8">
         <v>16</v>
       </c>
-      <c r="O83" s="8"/>
+      <c r="O83" s="8">
+        <f>AVERAGE(H83,N83)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" s="9">
@@ -5321,7 +5567,10 @@
       <c r="N84" s="1">
         <v>16</v>
       </c>
-      <c r="O84" s="1"/>
+      <c r="O84" s="1">
+        <f>AVERAGE(H84,N84)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" s="7">
@@ -5366,7 +5615,10 @@
       <c r="N85" s="8">
         <v>14</v>
       </c>
-      <c r="O85" s="8"/>
+      <c r="O85" s="8">
+        <f>AVERAGE(H85,N85)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" s="9">
@@ -5411,7 +5663,10 @@
       <c r="N86" s="1">
         <v>10</v>
       </c>
-      <c r="O86" s="1"/>
+      <c r="O86" s="1">
+        <f>AVERAGE(H86,N86)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87" s="7">
@@ -5456,7 +5711,10 @@
       <c r="N87" s="8">
         <v>17</v>
       </c>
-      <c r="O87" s="8"/>
+      <c r="O87" s="8">
+        <f>AVERAGE(H87,N87)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" s="9">
@@ -5501,7 +5759,10 @@
       <c r="N88" s="1">
         <v>9</v>
       </c>
-      <c r="O88" s="1"/>
+      <c r="O88" s="1">
+        <f>AVERAGE(H88,N88)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" s="7">
@@ -5546,7 +5807,10 @@
       <c r="N89" s="8">
         <v>19</v>
       </c>
-      <c r="O89" s="8"/>
+      <c r="O89" s="8">
+        <f>AVERAGE(H89,N89)</f>
+        <v>17.5</v>
+      </c>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90" s="9">
@@ -5591,7 +5855,10 @@
       <c r="N90" s="1">
         <v>10</v>
       </c>
-      <c r="O90" s="1"/>
+      <c r="O90" s="1">
+        <f>AVERAGE(H90,N90)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91" s="7">
@@ -5636,7 +5903,10 @@
       <c r="N91" s="8">
         <v>16</v>
       </c>
-      <c r="O91" s="8"/>
+      <c r="O91" s="8">
+        <f>AVERAGE(H91,N91)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92" s="9">
@@ -5681,7 +5951,10 @@
       <c r="N92" s="1">
         <v>17</v>
       </c>
-      <c r="O92" s="1"/>
+      <c r="O92" s="1">
+        <f>AVERAGE(H92,N92)</f>
+        <v>17.5</v>
+      </c>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93" s="7">
@@ -5726,7 +5999,10 @@
       <c r="N93" s="8">
         <v>18</v>
       </c>
-      <c r="O93" s="8"/>
+      <c r="O93" s="8">
+        <f>AVERAGE(H93,N93)</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94" s="9">
@@ -5771,7 +6047,10 @@
       <c r="N94" s="1">
         <v>14</v>
       </c>
-      <c r="O94" s="1"/>
+      <c r="O94" s="1">
+        <f>AVERAGE(H94,N94)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95" s="7">
@@ -5816,7 +6095,10 @@
       <c r="N95" s="8">
         <v>14</v>
       </c>
-      <c r="O95" s="8"/>
+      <c r="O95" s="8">
+        <f>AVERAGE(H95,N95)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96" s="9">
@@ -5861,7 +6143,10 @@
       <c r="N96" s="1">
         <v>12</v>
       </c>
-      <c r="O96" s="1"/>
+      <c r="O96" s="1">
+        <f>AVERAGE(H96,N96)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97" s="7">
@@ -5906,7 +6191,10 @@
       <c r="N97" s="8">
         <v>8</v>
       </c>
-      <c r="O97" s="8"/>
+      <c r="O97" s="8">
+        <f>AVERAGE(H97,N97)</f>
+        <v>8.5</v>
+      </c>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98" s="9">
@@ -5951,7 +6239,10 @@
       <c r="N98" s="1">
         <v>19</v>
       </c>
-      <c r="O98" s="1"/>
+      <c r="O98" s="1">
+        <f>AVERAGE(H98,N98)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" s="7">
@@ -5996,7 +6287,10 @@
       <c r="N99" s="8">
         <v>9</v>
       </c>
-      <c r="O99" s="8"/>
+      <c r="O99" s="8">
+        <f>AVERAGE(H99,N99)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" s="9">
@@ -6041,7 +6335,10 @@
       <c r="N100" s="1">
         <v>9</v>
       </c>
-      <c r="O100" s="1"/>
+      <c r="O100" s="1">
+        <f>AVERAGE(H100,N100)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" s="7">
@@ -6086,7 +6383,10 @@
       <c r="N101" s="8">
         <v>15</v>
       </c>
-      <c r="O101" s="8"/>
+      <c r="O101" s="8">
+        <f>AVERAGE(H101,N101)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" s="9">
@@ -6131,7 +6431,10 @@
       <c r="N102" s="1">
         <v>8</v>
       </c>
-      <c r="O102" s="1"/>
+      <c r="O102" s="1">
+        <f>AVERAGE(H102,N102)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" s="7">
@@ -6176,7 +6479,10 @@
       <c r="N103" s="8">
         <v>12</v>
       </c>
-      <c r="O103" s="8"/>
+      <c r="O103" s="8">
+        <f>AVERAGE(H103,N103)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" s="9">
@@ -6221,7 +6527,10 @@
       <c r="N104" s="1">
         <v>15</v>
       </c>
-      <c r="O104" s="1"/>
+      <c r="O104" s="1">
+        <f>AVERAGE(H104,N104)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" s="7">
@@ -6266,7 +6575,10 @@
       <c r="N105" s="8">
         <v>11</v>
       </c>
-      <c r="O105" s="8"/>
+      <c r="O105" s="8">
+        <f>AVERAGE(H105,N105)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="9">
@@ -6311,7 +6623,10 @@
       <c r="N106" s="1">
         <v>7</v>
       </c>
-      <c r="O106" s="1"/>
+      <c r="O106" s="1">
+        <f>AVERAGE(H106,N106)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="7">
@@ -6356,7 +6671,10 @@
       <c r="N107" s="8">
         <v>18</v>
       </c>
-      <c r="O107" s="8"/>
+      <c r="O107" s="8">
+        <f>AVERAGE(H107,N107)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="9">
@@ -6401,7 +6719,10 @@
       <c r="N108" s="1">
         <v>9</v>
       </c>
-      <c r="O108" s="1"/>
+      <c r="O108" s="1">
+        <f>AVERAGE(H108,N108)</f>
+        <v>8.5</v>
+      </c>
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="7">
@@ -6446,7 +6767,10 @@
       <c r="N109" s="8">
         <v>12</v>
       </c>
-      <c r="O109" s="8"/>
+      <c r="O109" s="8">
+        <f>AVERAGE(H109,N109)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="9">
@@ -6491,7 +6815,10 @@
       <c r="N110" s="1">
         <v>12</v>
       </c>
-      <c r="O110" s="1"/>
+      <c r="O110" s="1">
+        <f>AVERAGE(H110,N110)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="7">
@@ -6536,7 +6863,10 @@
       <c r="N111" s="8">
         <v>7</v>
       </c>
-      <c r="O111" s="8"/>
+      <c r="O111" s="8">
+        <f>AVERAGE(H111,N111)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="9">
@@ -6581,7 +6911,10 @@
       <c r="N112" s="1">
         <v>15</v>
       </c>
-      <c r="O112" s="1"/>
+      <c r="O112" s="1">
+        <f>AVERAGE(H112,N112)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" s="7">
@@ -6626,7 +6959,10 @@
       <c r="N113" s="8">
         <v>8</v>
       </c>
-      <c r="O113" s="8"/>
+      <c r="O113" s="8">
+        <f>AVERAGE(H113,N113)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" s="9">
@@ -6671,7 +7007,10 @@
       <c r="N114" s="1">
         <v>8</v>
       </c>
-      <c r="O114" s="1"/>
+      <c r="O114" s="1">
+        <f>AVERAGE(H114,N114)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" s="7">
@@ -6716,7 +7055,10 @@
       <c r="N115" s="8">
         <v>7</v>
       </c>
-      <c r="O115" s="8"/>
+      <c r="O115" s="8">
+        <f>AVERAGE(H115,N115)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" s="9">
@@ -6761,7 +7103,10 @@
       <c r="N116" s="1">
         <v>10</v>
       </c>
-      <c r="O116" s="1"/>
+      <c r="O116" s="1">
+        <f>AVERAGE(H116,N116)</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" s="7">
@@ -6806,7 +7151,10 @@
       <c r="N117" s="8">
         <v>15</v>
       </c>
-      <c r="O117" s="8"/>
+      <c r="O117" s="8">
+        <f>AVERAGE(H117,N117)</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" s="9">
@@ -6851,7 +7199,10 @@
       <c r="N118" s="1">
         <v>18</v>
       </c>
-      <c r="O118" s="1"/>
+      <c r="O118" s="1">
+        <f>AVERAGE(H118,N118)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" s="7">
@@ -6896,7 +7247,10 @@
       <c r="N119" s="8">
         <v>15</v>
       </c>
-      <c r="O119" s="8"/>
+      <c r="O119" s="8">
+        <f>AVERAGE(H119,N119)</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120" s="9">
@@ -6941,7 +7295,10 @@
       <c r="N120" s="1">
         <v>11</v>
       </c>
-      <c r="O120" s="1"/>
+      <c r="O120" s="1">
+        <f>AVERAGE(H120,N120)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121" s="7">
@@ -6986,7 +7343,10 @@
       <c r="N121" s="8">
         <v>11</v>
       </c>
-      <c r="O121" s="8"/>
+      <c r="O121" s="8">
+        <f>AVERAGE(H121,N121)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122" s="9">
@@ -7031,7 +7391,10 @@
       <c r="N122" s="1">
         <v>7</v>
       </c>
-      <c r="O122" s="1"/>
+      <c r="O122" s="1">
+        <f>AVERAGE(H122,N122)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123" s="7">
@@ -7076,7 +7439,10 @@
       <c r="N123" s="8">
         <v>16</v>
       </c>
-      <c r="O123" s="8"/>
+      <c r="O123" s="8">
+        <f>AVERAGE(H123,N123)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" s="9">
@@ -7121,7 +7487,10 @@
       <c r="N124" s="1">
         <v>10</v>
       </c>
-      <c r="O124" s="1"/>
+      <c r="O124" s="1">
+        <f>AVERAGE(H124,N124)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" s="7">
@@ -7166,7 +7535,10 @@
       <c r="N125" s="8">
         <v>14</v>
       </c>
-      <c r="O125" s="8"/>
+      <c r="O125" s="8">
+        <f>AVERAGE(H125,N125)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126" s="9">
@@ -7211,7 +7583,10 @@
       <c r="N126" s="1">
         <v>19</v>
       </c>
-      <c r="O126" s="1"/>
+      <c r="O126" s="1">
+        <f>AVERAGE(H126,N126)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127" s="7">
@@ -7256,7 +7631,10 @@
       <c r="N127" s="8">
         <v>10</v>
       </c>
-      <c r="O127" s="8"/>
+      <c r="O127" s="8">
+        <f>AVERAGE(H127,N127)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128" s="9">
@@ -7301,7 +7679,10 @@
       <c r="N128" s="1">
         <v>9</v>
       </c>
-      <c r="O128" s="1"/>
+      <c r="O128" s="1">
+        <f>AVERAGE(H128,N128)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A129" s="7">
@@ -7346,7 +7727,10 @@
       <c r="N129" s="8">
         <v>8</v>
       </c>
-      <c r="O129" s="8"/>
+      <c r="O129" s="8">
+        <f>AVERAGE(H129,N129)</f>
+        <v>8.5</v>
+      </c>
     </row>
     <row r="130" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A130" s="9">
@@ -7391,7 +7775,10 @@
       <c r="N130" s="1">
         <v>8</v>
       </c>
-      <c r="O130" s="1"/>
+      <c r="O130" s="1">
+        <f>AVERAGE(H130,N130)</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="131" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A131" s="7">
@@ -7436,7 +7823,10 @@
       <c r="N131" s="8">
         <v>9</v>
       </c>
-      <c r="O131" s="8"/>
+      <c r="O131" s="8">
+        <f>AVERAGE(H131,N131)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="132" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A132" s="9">
@@ -7481,7 +7871,10 @@
       <c r="N132" s="1">
         <v>8</v>
       </c>
-      <c r="O132" s="1"/>
+      <c r="O132" s="1">
+        <f>AVERAGE(H132,N132)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133" s="7">
@@ -7526,7 +7919,10 @@
       <c r="N133" s="8">
         <v>11</v>
       </c>
-      <c r="O133" s="8"/>
+      <c r="O133" s="8">
+        <f>AVERAGE(H133,N133)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134" s="9">
@@ -7571,7 +7967,10 @@
       <c r="N134" s="1">
         <v>9</v>
       </c>
-      <c r="O134" s="1"/>
+      <c r="O134" s="1">
+        <f>AVERAGE(H134,N134)</f>
+        <v>10.5</v>
+      </c>
     </row>
     <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135" s="7">
@@ -7616,7 +8015,10 @@
       <c r="N135" s="8">
         <v>12</v>
       </c>
-      <c r="O135" s="8"/>
+      <c r="O135" s="8">
+        <f>AVERAGE(H135,N135)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136" s="9">
@@ -7661,7 +8063,10 @@
       <c r="N136" s="1">
         <v>12</v>
       </c>
-      <c r="O136" s="1"/>
+      <c r="O136" s="1">
+        <f>AVERAGE(H136,N136)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137" s="7">
@@ -7706,7 +8111,10 @@
       <c r="N137" s="8">
         <v>19</v>
       </c>
-      <c r="O137" s="8"/>
+      <c r="O137" s="8">
+        <f>AVERAGE(H137,N137)</f>
+        <v>17.5</v>
+      </c>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138" s="9">
@@ -7751,7 +8159,10 @@
       <c r="N138" s="1">
         <v>19</v>
       </c>
-      <c r="O138" s="1"/>
+      <c r="O138" s="1">
+        <f>AVERAGE(H138,N138)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139" s="7">
@@ -7796,7 +8207,10 @@
       <c r="N139" s="8">
         <v>12</v>
       </c>
-      <c r="O139" s="8"/>
+      <c r="O139" s="8">
+        <f>AVERAGE(H139,N139)</f>
+        <v>11.5</v>
+      </c>
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140" s="9">
@@ -7841,7 +8255,10 @@
       <c r="N140" s="1">
         <v>9</v>
       </c>
-      <c r="O140" s="1"/>
+      <c r="O140" s="1">
+        <f>AVERAGE(H140,N140)</f>
+        <v>8.5</v>
+      </c>
     </row>
     <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141" s="7">
@@ -7886,7 +8303,10 @@
       <c r="N141" s="8">
         <v>18</v>
       </c>
-      <c r="O141" s="8"/>
+      <c r="O141" s="8">
+        <f>AVERAGE(H141,N141)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142" s="9">
@@ -7931,7 +8351,10 @@
       <c r="N142" s="1">
         <v>12</v>
       </c>
-      <c r="O142" s="1"/>
+      <c r="O142" s="1">
+        <f>AVERAGE(H142,N142)</f>
+        <v>13</v>
+      </c>
     </row>
     <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143" s="7">
@@ -7976,7 +8399,10 @@
       <c r="N143" s="8">
         <v>14</v>
       </c>
-      <c r="O143" s="8"/>
+      <c r="O143" s="8">
+        <f>AVERAGE(H143,N143)</f>
+        <v>11</v>
+      </c>
     </row>
     <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144" s="9">
@@ -8021,7 +8447,10 @@
       <c r="N144" s="1">
         <v>14</v>
       </c>
-      <c r="O144" s="1"/>
+      <c r="O144" s="1">
+        <f>AVERAGE(H144,N144)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="145" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A145" s="7">
@@ -8066,7 +8495,10 @@
       <c r="N145" s="8">
         <v>18</v>
       </c>
-      <c r="O145" s="8"/>
+      <c r="O145" s="8">
+        <f>AVERAGE(H145,N145)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="146" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A146" s="9">
@@ -8111,7 +8543,10 @@
       <c r="N146" s="1">
         <v>13</v>
       </c>
-      <c r="O146" s="1"/>
+      <c r="O146" s="1">
+        <f>AVERAGE(H146,N146)</f>
+        <v>15.5</v>
+      </c>
     </row>
     <row r="147" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A147" s="7">
@@ -8156,7 +8591,10 @@
       <c r="N147" s="8">
         <v>8</v>
       </c>
-      <c r="O147" s="8"/>
+      <c r="O147" s="8">
+        <f>AVERAGE(H147,N147)</f>
+        <v>9.5</v>
+      </c>
     </row>
     <row r="148" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A148" s="9">
@@ -8201,7 +8639,10 @@
       <c r="N148" s="1">
         <v>13</v>
       </c>
-      <c r="O148" s="1"/>
+      <c r="O148" s="1">
+        <f>AVERAGE(H148,N148)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A149" s="7">
@@ -8246,7 +8687,10 @@
       <c r="N149" s="8">
         <v>14</v>
       </c>
-      <c r="O149" s="8"/>
+      <c r="O149" s="8">
+        <f>AVERAGE(H149,N149)</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="150" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A150" s="9">
@@ -8291,7 +8735,10 @@
       <c r="N150" s="1">
         <v>9</v>
       </c>
-      <c r="O150" s="1"/>
+      <c r="O150" s="1">
+        <f>AVERAGE(H150,N150)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="151" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A151" s="7">
@@ -8336,7 +8783,10 @@
       <c r="N151" s="8">
         <v>19</v>
       </c>
-      <c r="O151" s="8"/>
+      <c r="O151" s="8">
+        <f>AVERAGE(H151,N151)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="152" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A152" s="9">
@@ -8381,7 +8831,10 @@
       <c r="N152" s="1">
         <v>18</v>
       </c>
-      <c r="O152" s="1"/>
+      <c r="O152" s="1">
+        <f>AVERAGE(H152,N152)</f>
+        <v>14.5</v>
+      </c>
     </row>
     <row r="153" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A153" s="7">
@@ -8426,7 +8879,10 @@
       <c r="N153" s="8">
         <v>10</v>
       </c>
-      <c r="O153" s="8"/>
+      <c r="O153" s="8">
+        <f>AVERAGE(H153,N153)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="154" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A154" s="9">
@@ -8471,7 +8927,10 @@
       <c r="N154" s="1">
         <v>8</v>
       </c>
-      <c r="O154" s="1"/>
+      <c r="O154" s="1">
+        <f>AVERAGE(H154,N154)</f>
+        <v>8</v>
+      </c>
     </row>
     <row r="155" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A155" s="7">
@@ -8516,7 +8975,10 @@
       <c r="N155" s="8">
         <v>16</v>
       </c>
-      <c r="O155" s="8"/>
+      <c r="O155" s="8">
+        <f>AVERAGE(H155,N155)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="156" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A156" s="9">
@@ -8561,7 +9023,10 @@
       <c r="N156" s="1">
         <v>12</v>
       </c>
-      <c r="O156" s="1"/>
+      <c r="O156" s="1">
+        <f>AVERAGE(H156,N156)</f>
+        <v>14</v>
+      </c>
     </row>
     <row r="157" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A157" s="7">
@@ -8606,7 +9071,10 @@
       <c r="N157" s="8">
         <v>16</v>
       </c>
-      <c r="O157" s="8"/>
+      <c r="O157" s="8">
+        <f>AVERAGE(H157,N157)</f>
+        <v>13.5</v>
+      </c>
     </row>
     <row r="158" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A158" s="9">
@@ -8651,7 +9119,10 @@
       <c r="N158" s="1">
         <v>16</v>
       </c>
-      <c r="O158" s="1"/>
+      <c r="O158" s="1">
+        <f>AVERAGE(H158,N158)</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="159" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A159" s="7">
@@ -8696,7 +9167,10 @@
       <c r="N159" s="8">
         <v>15</v>
       </c>
-      <c r="O159" s="8"/>
+      <c r="O159" s="8">
+        <f>AVERAGE(H159,N159)</f>
+        <v>12.5</v>
+      </c>
     </row>
     <row r="160" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A160" s="9">
@@ -8741,7 +9215,10 @@
       <c r="N160" s="1">
         <v>7</v>
       </c>
-      <c r="O160" s="1"/>
+      <c r="O160" s="1">
+        <f>AVERAGE(H160,N160)</f>
+        <v>8.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>